<commit_message>
threhsold clean and skadi data added
</commit_message>
<xml_diff>
--- a/config/MB300L_thresholds.xlsx
+++ b/config/MB300L_thresholds.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/francescopiscitelli/git_repos/mbuty/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90AB5D14-1477-3A4D-ACD6-9AA3CFE8749C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3F9F0A1-228E-6F48-8A21-B5F8D1679EB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-39560" yWindow="600" windowWidth="37540" windowHeight="26360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -488,7 +488,7 @@
         <v>5000</v>
       </c>
       <c r="G2" s="3">
-        <v>7000</v>
+        <v>1200</v>
       </c>
       <c r="H2" s="3">
         <v>10500</v>
@@ -514,7 +514,7 @@
         <v>15000</v>
       </c>
       <c r="G3" s="3">
-        <v>7000</v>
+        <v>1200</v>
       </c>
       <c r="H3" s="3">
         <v>18500</v>
@@ -540,7 +540,7 @@
         <v>14000</v>
       </c>
       <c r="G4" s="3">
-        <v>7000</v>
+        <v>1200</v>
       </c>
       <c r="H4" s="3">
         <v>19500</v>
@@ -566,7 +566,7 @@
         <v>15000</v>
       </c>
       <c r="G5" s="3">
-        <v>7000</v>
+        <v>1200</v>
       </c>
       <c r="H5" s="3">
         <v>19500</v>
@@ -592,7 +592,7 @@
         <v>16000</v>
       </c>
       <c r="G6" s="3">
-        <v>7000</v>
+        <v>1200</v>
       </c>
       <c r="H6" s="3">
         <v>21500</v>
@@ -618,7 +618,7 @@
         <v>10000</v>
       </c>
       <c r="G7" s="3">
-        <v>7000</v>
+        <v>1200</v>
       </c>
       <c r="H7" s="3">
         <v>15000</v>
@@ -644,7 +644,7 @@
         <v>15000</v>
       </c>
       <c r="G8" s="3">
-        <v>12195.121951219511</v>
+        <v>500</v>
       </c>
       <c r="H8" s="3">
         <v>19744.483159117302</v>
@@ -670,7 +670,7 @@
         <v>17000</v>
       </c>
       <c r="G9" s="3">
-        <v>11904.761904761903</v>
+        <v>500</v>
       </c>
       <c r="H9" s="3">
         <v>19274.376417233558</v>
@@ -696,7 +696,7 @@
         <v>16279.069767441859</v>
       </c>
       <c r="G10" s="3">
-        <v>11627.906976744185</v>
+        <v>500</v>
       </c>
       <c r="H10" s="3">
         <v>18826.13510520487</v>
@@ -722,7 +722,7 @@
         <v>15909.09090909091</v>
       </c>
       <c r="G11" s="3">
-        <v>11363.636363636364</v>
+        <v>500</v>
       </c>
       <c r="H11" s="3">
         <v>18398.268398268399</v>
@@ -748,7 +748,7 @@
         <v>15555.555555555555</v>
       </c>
       <c r="G12" s="3">
-        <v>11111.111111111111</v>
+        <v>500</v>
       </c>
       <c r="H12" s="3">
         <v>18888.888888888887</v>
@@ -774,7 +774,7 @@
         <v>15217.391304347826</v>
       </c>
       <c r="G13" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H13" s="3">
         <v>18478.260869565216</v>
@@ -800,7 +800,7 @@
         <v>14893.617021276596</v>
       </c>
       <c r="G14" s="3">
-        <v>14000</v>
+        <v>500</v>
       </c>
       <c r="H14" s="3">
         <v>18500</v>
@@ -826,7 +826,7 @@
         <v>15500</v>
       </c>
       <c r="G15" s="3">
-        <v>14000</v>
+        <v>500</v>
       </c>
       <c r="H15" s="3">
         <v>18500</v>
@@ -852,7 +852,7 @@
         <v>14285.714285714286</v>
       </c>
       <c r="G16" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H16" s="3">
         <v>16500</v>
@@ -878,7 +878,7 @@
         <v>13000</v>
       </c>
       <c r="G17" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H17" s="3">
         <v>18000</v>
@@ -904,7 +904,7 @@
         <v>13725.490196078432</v>
       </c>
       <c r="G18" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H18" s="3">
         <v>17000</v>
@@ -930,7 +930,7 @@
         <v>13461.538461538461</v>
       </c>
       <c r="G19" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H19" s="3">
         <v>15000</v>
@@ -956,7 +956,7 @@
         <v>13207.54716981132</v>
       </c>
       <c r="G20" s="3">
-        <v>12500</v>
+        <v>500</v>
       </c>
       <c r="H20" s="3">
         <v>15000</v>
@@ -982,7 +982,7 @@
         <v>14000</v>
       </c>
       <c r="G21" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H21" s="3">
         <v>15500</v>
@@ -1008,7 +1008,7 @@
         <v>12727.272727272726</v>
       </c>
       <c r="G22" s="3">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="H22" s="3">
         <v>18500</v>
@@ -1034,7 +1034,7 @@
         <v>12499.999999999998</v>
       </c>
       <c r="G23" s="3">
-        <v>12500</v>
+        <v>500</v>
       </c>
       <c r="H23" s="3">
         <v>15178.571428571428</v>
@@ -1060,7 +1060,7 @@
         <v>12280.701754385964</v>
       </c>
       <c r="G24" s="3">
-        <v>11000</v>
+        <v>0</v>
       </c>
       <c r="H24" s="3">
         <v>13000</v>
@@ -1086,7 +1086,7 @@
         <v>12068.965517241379</v>
       </c>
       <c r="G25" s="3">
-        <v>12500</v>
+        <v>500</v>
       </c>
       <c r="H25" s="3">
         <v>13500</v>
@@ -1112,7 +1112,7 @@
         <v>11864.406779661016</v>
       </c>
       <c r="G26" s="3">
-        <v>12000</v>
+        <v>500</v>
       </c>
       <c r="H26" s="3">
         <v>14406.779661016948</v>
@@ -1138,7 +1138,7 @@
         <v>11666.666666666664</v>
       </c>
       <c r="G27" s="3">
-        <v>13000</v>
+        <v>1000</v>
       </c>
       <c r="H27" s="3">
         <v>14166.666666666664</v>
@@ -1164,7 +1164,7 @@
         <v>11475.409836065573</v>
       </c>
       <c r="G28" s="3">
-        <v>9000</v>
+        <v>500</v>
       </c>
       <c r="H28" s="3">
         <v>15000</v>
@@ -1190,7 +1190,7 @@
         <v>11290.322580645161</v>
       </c>
       <c r="G29" s="3">
-        <v>9000</v>
+        <v>500</v>
       </c>
       <c r="H29" s="3">
         <v>13709.677419354839</v>
@@ -1216,7 +1216,7 @@
         <v>11111.111111111111</v>
       </c>
       <c r="G30" s="3">
-        <v>9000</v>
+        <v>500</v>
       </c>
       <c r="H30" s="3">
         <v>13492.063492063491</v>
@@ -1242,7 +1242,7 @@
         <v>10937.5</v>
       </c>
       <c r="G31" s="3">
-        <v>9000</v>
+        <v>500</v>
       </c>
       <c r="H31" s="3">
         <v>13281.25</v>
@@ -1268,7 +1268,7 @@
         <v>10769.23076923077</v>
       </c>
       <c r="G32" s="3">
-        <v>9000</v>
+        <v>500</v>
       </c>
       <c r="H32" s="3">
         <v>13076.923076923076</v>
@@ -1294,7 +1294,7 @@
         <v>20000</v>
       </c>
       <c r="G33" s="3">
-        <v>20000</v>
+        <v>500</v>
       </c>
       <c r="H33" s="3">
         <v>20000</v>

</xml_diff>